<commit_message>
feat: implement SOP editor component with reactive form logic, inventory/recipe integration, and dynamic target configuration
</commit_message>
<xml_diff>
--- a/LIMS_Master_Analytes.xlsx
+++ b/LIMS_Master_Analytes.xlsx
@@ -397,14 +397,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F136"/>
+  <dimension ref="A1:F166"/>
   <cols>
-    <col min="1" max="1" width="35.83203125" customWidth="1"/>
+    <col min="1" max="1" width="39.83203125" customWidth="1"/>
     <col min="2" max="2" width="39.83203125" customWidth="1"/>
     <col min="3" max="3" width="13.83203125" customWidth="1"/>
     <col min="4" max="4" width="20.83203125" customWidth="1"/>
     <col min="5" max="5" width="18.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+    <col min="6" max="6" width="29.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -429,10 +429,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>acephate</v>
+        <v>1_naphthol</v>
       </c>
       <c r="B2" t="str">
-        <v>Acephate</v>
+        <v>1-Naphthol</v>
       </c>
       <c r="C2" t="str">
         <v/>
@@ -444,15 +444,15 @@
         <v>ppb</v>
       </c>
       <c r="F2" t="str">
-        <v/>
+        <v>SOP 9.14 USDA</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>alachlor</v>
+        <v>acephate</v>
       </c>
       <c r="B3" t="str">
-        <v>Alachlor</v>
+        <v>Acephate</v>
       </c>
       <c r="C3" t="str">
         <v/>
@@ -469,10 +469,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>aldrin</v>
+        <v>acetamiprid</v>
       </c>
       <c r="B4" t="str">
-        <v>Aldrin</v>
+        <v>Acetamiprid</v>
       </c>
       <c r="C4" t="str">
         <v/>
@@ -484,15 +484,15 @@
         <v>ppb</v>
       </c>
       <c r="F4" t="str">
-        <v/>
+        <v>SOP 9.14 USDA</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>atrazine</v>
+        <v>alachlor</v>
       </c>
       <c r="B5" t="str">
-        <v>Atrazine</v>
+        <v>Alachlor</v>
       </c>
       <c r="C5" t="str">
         <v/>
@@ -509,10 +509,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>azinphos_methyl</v>
+        <v>aldrin</v>
       </c>
       <c r="B6" t="str">
-        <v>Azinphos-methyl</v>
+        <v>Aldrin</v>
       </c>
       <c r="C6" t="str">
         <v/>
@@ -529,10 +529,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>azoxystrobin</v>
+        <v>atrazine</v>
       </c>
       <c r="B7" t="str">
-        <v>Azoxystrobin</v>
+        <v>Atrazine</v>
       </c>
       <c r="C7" t="str">
         <v/>
@@ -549,10 +549,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>fat_total</v>
+        <v>azinphos_methyl</v>
       </c>
       <c r="B8" t="str">
-        <v>Béo tổng (Total Fat as Triglyceride)</v>
+        <v>Azinphos-methyl</v>
       </c>
       <c r="C8" t="str">
         <v/>
@@ -561,7 +561,7 @@
         <v/>
       </c>
       <c r="E8" t="str">
-        <v>g/100g</v>
+        <v>ppb</v>
       </c>
       <c r="F8" t="str">
         <v/>
@@ -569,10 +569,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>bhc_alpha_benzene_hexachloride</v>
+        <v>azinfos_methyl</v>
       </c>
       <c r="B9" t="str">
-        <v>BHC-alpha (benzene hexachloride)</v>
+        <v>Azinphos-methyl</v>
       </c>
       <c r="C9" t="str">
         <v/>
@@ -589,10 +589,10 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>bhc_beta</v>
+        <v>azoxystrobin</v>
       </c>
       <c r="B10" t="str">
-        <v>BHC-beta</v>
+        <v>Azoxystrobin</v>
       </c>
       <c r="C10" t="str">
         <v/>
@@ -609,10 +609,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>bhc_delta</v>
+        <v>béo_tổng_(total_fat_as_triglyceride)</v>
       </c>
       <c r="B11" t="str">
-        <v>BHC-delta</v>
+        <v>Béo tổng (Total Fat as Triglyceride)</v>
       </c>
       <c r="C11" t="str">
         <v/>
@@ -621,7 +621,7 @@
         <v/>
       </c>
       <c r="E11" t="str">
-        <v>ppb</v>
+        <v>g/100g</v>
       </c>
       <c r="F11" t="str">
         <v/>
@@ -629,10 +629,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>bhc_epsilon</v>
+        <v>fat_total</v>
       </c>
       <c r="B12" t="str">
-        <v>BHC-epsilon</v>
+        <v>Béo tổng (Total Fat as Triglyceride)</v>
       </c>
       <c r="C12" t="str">
         <v/>
@@ -641,7 +641,7 @@
         <v/>
       </c>
       <c r="E12" t="str">
-        <v>ppb</v>
+        <v>g/100g</v>
       </c>
       <c r="F12" t="str">
         <v/>
@@ -649,10 +649,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>bhc_gamma_lindane_gamma_hch</v>
+        <v>bhc_alpha_benzene_hexachloride</v>
       </c>
       <c r="B13" t="str">
-        <v>BHC-gamma (Lindane, gamma HCH)</v>
+        <v>BHC-alpha (benzene hexachloride)</v>
       </c>
       <c r="C13" t="str">
         <v/>
@@ -669,10 +669,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>bifenthrin</v>
+        <v>bhc_beta</v>
       </c>
       <c r="B14" t="str">
-        <v>Bifenthrin</v>
+        <v>BHC-beta</v>
       </c>
       <c r="C14" t="str">
         <v/>
@@ -689,10 +689,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>bitertanol</v>
+        <v>bhc_delta</v>
       </c>
       <c r="B15" t="str">
-        <v>Bitertanol</v>
+        <v>BHC-delta</v>
       </c>
       <c r="C15" t="str">
         <v/>
@@ -709,10 +709,10 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>boscalid</v>
+        <v>bhc_epsilon</v>
       </c>
       <c r="B16" t="str">
-        <v>Boscalid</v>
+        <v>BHC-epsilon</v>
       </c>
       <c r="C16" t="str">
         <v/>
@@ -729,10 +729,10 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>buprofezin</v>
+        <v>bhc_gamma_lindane_gamma_hch</v>
       </c>
       <c r="B17" t="str">
-        <v>Buprofezin</v>
+        <v>BHC-gamma (Lindane, gamma HCH)</v>
       </c>
       <c r="C17" t="str">
         <v/>
@@ -749,10 +749,10 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>butachlor</v>
+        <v>bifenthrin</v>
       </c>
       <c r="B18" t="str">
-        <v>Butachlor</v>
+        <v>Bifenthrin</v>
       </c>
       <c r="C18" t="str">
         <v/>
@@ -769,10 +769,10 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>cadusafos</v>
+        <v>bitertanol</v>
       </c>
       <c r="B19" t="str">
-        <v>Cadusafos</v>
+        <v>Bitertanol</v>
       </c>
       <c r="C19" t="str">
         <v/>
@@ -789,10 +789,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>chlordane_cis_alpha</v>
+        <v>boscalid</v>
       </c>
       <c r="B20" t="str">
-        <v>Chlordane-cis (alpha)</v>
+        <v>Boscalid</v>
       </c>
       <c r="C20" t="str">
         <v/>
@@ -809,10 +809,10 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>chlordane_oxy</v>
+        <v>buprofezin</v>
       </c>
       <c r="B21" t="str">
-        <v>Chlordane-oxy</v>
+        <v>Buprofezin</v>
       </c>
       <c r="C21" t="str">
         <v/>
@@ -829,10 +829,10 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>chlordane_trans_gamma</v>
+        <v>butachlor</v>
       </c>
       <c r="B22" t="str">
-        <v>Chlordane-trans (gamma)</v>
+        <v>Butachlor</v>
       </c>
       <c r="C22" t="str">
         <v/>
@@ -849,10 +849,10 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>chlorfenapyr</v>
+        <v>cadusafos</v>
       </c>
       <c r="B23" t="str">
-        <v>Chlorfenapyr</v>
+        <v>Cadusafos</v>
       </c>
       <c r="C23" t="str">
         <v/>
@@ -869,10 +869,10 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>chlorfenvinphos</v>
+        <v>chlordane_cis_alpha</v>
       </c>
       <c r="B24" t="str">
-        <v>Chlorfenvinphos</v>
+        <v>Chlordane-cis (alpha)</v>
       </c>
       <c r="C24" t="str">
         <v/>
@@ -889,10 +889,10 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>chlorothalonil</v>
+        <v>chlordane_oxy</v>
       </c>
       <c r="B25" t="str">
-        <v>Chlorothalonil</v>
+        <v>Chlordane-oxy</v>
       </c>
       <c r="C25" t="str">
         <v/>
@@ -909,10 +909,10 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>chlorpyrifos</v>
+        <v>chlordane_trans_gamma</v>
       </c>
       <c r="B26" t="str">
-        <v>Chlorpyrifos</v>
+        <v>Chlordane-trans (gamma)</v>
       </c>
       <c r="C26" t="str">
         <v/>
@@ -929,10 +929,10 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>chlorpyrifos_methyl</v>
+        <v>chlorfenapyr</v>
       </c>
       <c r="B27" t="str">
-        <v>Chlorpyrifos-methyl</v>
+        <v>Chlorfenapyr</v>
       </c>
       <c r="C27" t="str">
         <v/>
@@ -949,10 +949,10 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>chlorpyrifos_methyl_desmethyl</v>
+        <v>chlorfenvinphos</v>
       </c>
       <c r="B28" t="str">
-        <v>Chlorpyrifos-methyl-desmethyl</v>
+        <v>Chlorfenvinphos</v>
       </c>
       <c r="C28" t="str">
         <v/>
@@ -969,10 +969,10 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>cyfluthrin_baythroid</v>
+        <v>chloroform</v>
       </c>
       <c r="B29" t="str">
-        <v>Cyfluthrin (Baythroid)</v>
+        <v>Chloroform</v>
       </c>
       <c r="C29" t="str">
         <v/>
@@ -989,10 +989,10 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>cypermethrins</v>
+        <v>chloroneb</v>
       </c>
       <c r="B30" t="str">
-        <v>Cypermethrins</v>
+        <v>Chloroneb</v>
       </c>
       <c r="C30" t="str">
         <v/>
@@ -1004,15 +1004,15 @@
         <v>ppb</v>
       </c>
       <c r="F30" t="str">
-        <v/>
+        <v>SOP 9.14 USDA</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>cyproconazole</v>
+        <v>chlorothalonil</v>
       </c>
       <c r="B31" t="str">
-        <v>Cyproconazole</v>
+        <v>Chlorothalonil</v>
       </c>
       <c r="C31" t="str">
         <v/>
@@ -1029,10 +1029,10 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>cyprodinil</v>
+        <v>chlorpropham</v>
       </c>
       <c r="B32" t="str">
-        <v>Cyprodinil</v>
+        <v>Chlorpropham</v>
       </c>
       <c r="C32" t="str">
         <v/>
@@ -1044,15 +1044,15 @@
         <v>ppb</v>
       </c>
       <c r="F32" t="str">
-        <v/>
+        <v>SOP 9.14 USDA</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>ddd_op</v>
+        <v>chlorpyrifos</v>
       </c>
       <c r="B33" t="str">
-        <v>DDD-o,p'</v>
+        <v>Chlorpyrifos</v>
       </c>
       <c r="C33" t="str">
         <v/>
@@ -1069,10 +1069,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>ddd_pp</v>
+        <v>chlorpyrifos_methyl</v>
       </c>
       <c r="B34" t="str">
-        <v>DDD-p,p'</v>
+        <v>Chlorpyrifos-methyl</v>
       </c>
       <c r="C34" t="str">
         <v/>
@@ -1089,10 +1089,10 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>dde_op</v>
+        <v>chlorpyrifos_methyl_desmethyl</v>
       </c>
       <c r="B35" t="str">
-        <v>DDE-o,p'</v>
+        <v>Chlorpyrifos-methyl-desmethyl</v>
       </c>
       <c r="C35" t="str">
         <v/>
@@ -1109,10 +1109,10 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>dde_pp</v>
+        <v>cyfluthrin_baythroid</v>
       </c>
       <c r="B36" t="str">
-        <v>DDE-p,p'</v>
+        <v>Cyfluthrin (Baythroid)</v>
       </c>
       <c r="C36" t="str">
         <v/>
@@ -1129,10 +1129,10 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>ddt_op</v>
+        <v>cypermethrins</v>
       </c>
       <c r="B37" t="str">
-        <v>DDT-o,p'</v>
+        <v>Cypermethrins</v>
       </c>
       <c r="C37" t="str">
         <v/>
@@ -1149,10 +1149,10 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>ddt_pp</v>
+        <v>cypermethrin</v>
       </c>
       <c r="B38" t="str">
-        <v>DDT-p,p'</v>
+        <v>Cypermethrins</v>
       </c>
       <c r="C38" t="str">
         <v/>
@@ -1169,10 +1169,10 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>deltamethrin</v>
+        <v>cyproconazole</v>
       </c>
       <c r="B39" t="str">
-        <v>Deltamethrin</v>
+        <v>Cyproconazole</v>
       </c>
       <c r="C39" t="str">
         <v/>
@@ -1189,10 +1189,10 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>diazinon</v>
+        <v>cyprodinil</v>
       </c>
       <c r="B40" t="str">
-        <v>Diazinon</v>
+        <v>Cyprodinil</v>
       </c>
       <c r="C40" t="str">
         <v/>
@@ -1209,10 +1209,10 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>dicloran</v>
+        <v>ddd_o_p</v>
       </c>
       <c r="B41" t="str">
-        <v>Dicloran</v>
+        <v>DDD-o,p'</v>
       </c>
       <c r="C41" t="str">
         <v/>
@@ -1229,10 +1229,10 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>dieldrin</v>
+        <v>ddd_op</v>
       </c>
       <c r="B42" t="str">
-        <v>Dieldrin</v>
+        <v>DDD-o,p'</v>
       </c>
       <c r="C42" t="str">
         <v/>
@@ -1249,10 +1249,10 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>difenoconazole</v>
+        <v>ddd_p_p</v>
       </c>
       <c r="B43" t="str">
-        <v>Difenoconazole</v>
+        <v>DDD-p,p'</v>
       </c>
       <c r="C43" t="str">
         <v/>
@@ -1269,10 +1269,10 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>dimethoate</v>
+        <v>ddd_pp</v>
       </c>
       <c r="B44" t="str">
-        <v>Dimethoate</v>
+        <v>DDD-p,p'</v>
       </c>
       <c r="C44" t="str">
         <v/>
@@ -1289,10 +1289,10 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>edifenphos</v>
+        <v>dde_o_p</v>
       </c>
       <c r="B45" t="str">
-        <v>Edifenphos</v>
+        <v>DDE-o,p'</v>
       </c>
       <c r="C45" t="str">
         <v/>
@@ -1309,10 +1309,10 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>endosulfan_i_alpha_isomer</v>
+        <v>dde_op</v>
       </c>
       <c r="B46" t="str">
-        <v>Endosulfan I (alpha isomer)</v>
+        <v>DDE-o,p'</v>
       </c>
       <c r="C46" t="str">
         <v/>
@@ -1329,10 +1329,10 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>endosulfan_ii_beta_isomer</v>
+        <v>dde_p_p</v>
       </c>
       <c r="B47" t="str">
-        <v>Endosulfan II (beta isomer)</v>
+        <v>DDE-p,p'</v>
       </c>
       <c r="C47" t="str">
         <v/>
@@ -1349,10 +1349,10 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>endosulfan_sulfate</v>
+        <v>dde_pp</v>
       </c>
       <c r="B48" t="str">
-        <v>Endosulfan sulfate</v>
+        <v>DDE-p,p'</v>
       </c>
       <c r="C48" t="str">
         <v/>
@@ -1369,10 +1369,10 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>endrin</v>
+        <v>ddt_o_p</v>
       </c>
       <c r="B49" t="str">
-        <v>Endrin</v>
+        <v>DDT-o,p'</v>
       </c>
       <c r="C49" t="str">
         <v/>
@@ -1389,10 +1389,10 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>ethanol</v>
+        <v>ddt_op</v>
       </c>
       <c r="B50" t="str">
-        <v>Ethanol</v>
+        <v>DDT-o,p'</v>
       </c>
       <c r="C50" t="str">
         <v/>
@@ -1409,10 +1409,10 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>ethion</v>
+        <v>ddt_p_p</v>
       </c>
       <c r="B51" t="str">
-        <v>Ethion</v>
+        <v>DDT-p,p'</v>
       </c>
       <c r="C51" t="str">
         <v/>
@@ -1429,10 +1429,10 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>ethofenprox</v>
+        <v>ddt_pp</v>
       </c>
       <c r="B52" t="str">
-        <v>Ethofenprox</v>
+        <v>DDT-p,p'</v>
       </c>
       <c r="C52" t="str">
         <v/>
@@ -1449,10 +1449,10 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>ethoprophos_ethoprop</v>
+        <v>deltamethrin</v>
       </c>
       <c r="B53" t="str">
-        <v>Ethoprophos (Ethoprop)</v>
+        <v>Deltamethrin</v>
       </c>
       <c r="C53" t="str">
         <v/>
@@ -1469,10 +1469,10 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>fenbuconazole</v>
+        <v>diazinon</v>
       </c>
       <c r="B54" t="str">
-        <v>Fenbuconazole</v>
+        <v>Diazinon</v>
       </c>
       <c r="C54" t="str">
         <v/>
@@ -1489,10 +1489,10 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>fenitrothion</v>
+        <v>dichlorvos</v>
       </c>
       <c r="B55" t="str">
-        <v>Fenitrothion</v>
+        <v>Dichlorvos</v>
       </c>
       <c r="C55" t="str">
         <v/>
@@ -1504,15 +1504,15 @@
         <v>ppb</v>
       </c>
       <c r="F55" t="str">
-        <v/>
+        <v>SOP 9.14 USDA (Tach rieng)</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>fenoxanil</v>
+        <v>dicloran</v>
       </c>
       <c r="B56" t="str">
-        <v>Fenoxanil</v>
+        <v>Dicloran</v>
       </c>
       <c r="C56" t="str">
         <v/>
@@ -1529,10 +1529,10 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>fenpropathrin</v>
+        <v>dieldrin</v>
       </c>
       <c r="B57" t="str">
-        <v>Fenpropathrin</v>
+        <v>Dieldrin</v>
       </c>
       <c r="C57" t="str">
         <v/>
@@ -1549,10 +1549,10 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>fenthion</v>
+        <v>difenoconazole</v>
       </c>
       <c r="B58" t="str">
-        <v>Fenthion</v>
+        <v>Difenoconazole</v>
       </c>
       <c r="C58" t="str">
         <v/>
@@ -1569,10 +1569,10 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>fenvalerate</v>
+        <v>dimethoate</v>
       </c>
       <c r="B59" t="str">
-        <v>Fenvalerate</v>
+        <v>Dimethoate</v>
       </c>
       <c r="C59" t="str">
         <v/>
@@ -1589,10 +1589,10 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>fipronil_2</v>
+        <v>edifenphos</v>
       </c>
       <c r="B60" t="str">
-        <v>Fipronil</v>
+        <v>Edifenphos</v>
       </c>
       <c r="C60" t="str">
         <v/>
@@ -1609,10 +1609,10 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>fipronil</v>
+        <v>edifenfos</v>
       </c>
       <c r="B61" t="str">
-        <v>Fipronil</v>
+        <v>Edifenphos</v>
       </c>
       <c r="C61" t="str">
         <v/>
@@ -1629,10 +1629,10 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>fipronil_desulfinyl</v>
+        <v>endosulfan_i_alpha_isomer</v>
       </c>
       <c r="B62" t="str">
-        <v>Fipronil-desulfinyl</v>
+        <v>Endosulfan I (alpha isomer)</v>
       </c>
       <c r="C62" t="str">
         <v/>
@@ -1649,10 +1649,10 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>fipronil_sulfide</v>
+        <v>endosulfan_ii_beta_isomer</v>
       </c>
       <c r="B63" t="str">
-        <v>Fipronil-sulfide</v>
+        <v>Endosulfan II (beta isomer)</v>
       </c>
       <c r="C63" t="str">
         <v/>
@@ -1669,10 +1669,10 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>fipronil_sulfone</v>
+        <v>endosulfan_sulfate</v>
       </c>
       <c r="B64" t="str">
-        <v>Fipronil-sulfone</v>
+        <v>Endosulfan sulfate</v>
       </c>
       <c r="C64" t="str">
         <v/>
@@ -1689,10 +1689,10 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>fluazifop</v>
+        <v>endrin</v>
       </c>
       <c r="B65" t="str">
-        <v>Fluazifop</v>
+        <v>Endrin</v>
       </c>
       <c r="C65" t="str">
         <v/>
@@ -1709,10 +1709,10 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>flucythrinate</v>
+        <v>ethanol</v>
       </c>
       <c r="B66" t="str">
-        <v>Flucythrinate</v>
+        <v>Ethanol</v>
       </c>
       <c r="C66" t="str">
         <v/>
@@ -1729,10 +1729,10 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>fludioxonil</v>
+        <v>ethion</v>
       </c>
       <c r="B67" t="str">
-        <v>Fludioxonil</v>
+        <v>Ethion</v>
       </c>
       <c r="C67" t="str">
         <v/>
@@ -1749,10 +1749,10 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>flufenacet</v>
+        <v>ethofenprox</v>
       </c>
       <c r="B68" t="str">
-        <v>Flufenacet</v>
+        <v>Ethofenprox</v>
       </c>
       <c r="C68" t="str">
         <v/>
@@ -1769,10 +1769,10 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>flusilazole</v>
+        <v>ethoprophos_ethoprop</v>
       </c>
       <c r="B69" t="str">
-        <v>Flusilazole</v>
+        <v>Ethoprophos (Ethoprop)</v>
       </c>
       <c r="C69" t="str">
         <v/>
@@ -1789,10 +1789,10 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>flutriafol</v>
+        <v>fenbuconazole</v>
       </c>
       <c r="B70" t="str">
-        <v>Flutriafol</v>
+        <v>Fenbuconazole</v>
       </c>
       <c r="C70" t="str">
         <v/>
@@ -1809,10 +1809,10 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>heptachlor</v>
+        <v>fenitrothion</v>
       </c>
       <c r="B71" t="str">
-        <v>Heptachlor</v>
+        <v>Fenitrothion</v>
       </c>
       <c r="C71" t="str">
         <v/>
@@ -1829,10 +1829,10 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>heptachlor_endo_epoxide_isomer_a</v>
+        <v>fenoxanil</v>
       </c>
       <c r="B72" t="str">
-        <v>Heptachlor endo-epoxide (isomer A)</v>
+        <v>Fenoxanil</v>
       </c>
       <c r="C72" t="str">
         <v/>
@@ -1849,10 +1849,10 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>heptachlor_exo_epoxide_isomer_b</v>
+        <v>fenpropathrin</v>
       </c>
       <c r="B73" t="str">
-        <v>Heptachlor exo-epoxide (isomer B)</v>
+        <v>Fenpropathrin</v>
       </c>
       <c r="C73" t="str">
         <v/>
@@ -1869,10 +1869,10 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>hexachlorobenzene</v>
+        <v>fenthion</v>
       </c>
       <c r="B74" t="str">
-        <v>Hexachlorobenzene</v>
+        <v>Fenthion</v>
       </c>
       <c r="C74" t="str">
         <v/>
@@ -1889,10 +1889,10 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>hexaconazole</v>
+        <v>fenvalerate</v>
       </c>
       <c r="B75" t="str">
-        <v>Hexaconazole</v>
+        <v>Fenvalerate</v>
       </c>
       <c r="C75" t="str">
         <v/>
@@ -1909,10 +1909,10 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>imazalil</v>
+        <v>fipronil</v>
       </c>
       <c r="B76" t="str">
-        <v>Imazalil</v>
+        <v>Fipronil</v>
       </c>
       <c r="C76" t="str">
         <v/>
@@ -1929,10 +1929,10 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>iprobenfos</v>
+        <v>fipronil_2</v>
       </c>
       <c r="B77" t="str">
-        <v>Iprobenfos</v>
+        <v>Fipronil</v>
       </c>
       <c r="C77" t="str">
         <v/>
@@ -1949,10 +1949,10 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>isodrin</v>
+        <v>fipronil_desulfinyl</v>
       </c>
       <c r="B78" t="str">
-        <v>Isodrin</v>
+        <v>Fipronil-desulfinyl</v>
       </c>
       <c r="C78" t="str">
         <v/>
@@ -1969,10 +1969,10 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>isofenphos_methyl</v>
+        <v>fipronil_sulfide</v>
       </c>
       <c r="B79" t="str">
-        <v>Isofenphos methyl</v>
+        <v>Fipronil-sulfide</v>
       </c>
       <c r="C79" t="str">
         <v/>
@@ -1989,10 +1989,10 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>kresoxim_methyl</v>
+        <v>fipronil_sulfone</v>
       </c>
       <c r="B80" t="str">
-        <v>Kresoxim methyl</v>
+        <v>Fipronil-sulfone</v>
       </c>
       <c r="C80" t="str">
         <v/>
@@ -2009,10 +2009,10 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>lamda_cyhalothrin</v>
+        <v>fluazifop</v>
       </c>
       <c r="B81" t="str">
-        <v>lamda-Cyhalothrin</v>
+        <v>Fluazifop</v>
       </c>
       <c r="C81" t="str">
         <v/>
@@ -2029,10 +2029,10 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>malathion</v>
+        <v>flucythrinate</v>
       </c>
       <c r="B82" t="str">
-        <v>Malathion</v>
+        <v>Flucythrinate</v>
       </c>
       <c r="C82" t="str">
         <v/>
@@ -2049,10 +2049,10 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>mecarbam</v>
+        <v>fludioxonil</v>
       </c>
       <c r="B83" t="str">
-        <v>Mecarbam</v>
+        <v>Fludioxonil</v>
       </c>
       <c r="C83" t="str">
         <v/>
@@ -2069,10 +2069,10 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>mefenacet</v>
+        <v>flufenacet</v>
       </c>
       <c r="B84" t="str">
-        <v>Mefenacet</v>
+        <v>Flufenacet</v>
       </c>
       <c r="C84" t="str">
         <v/>
@@ -2089,10 +2089,10 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>mefenoxam</v>
+        <v>flusilazole</v>
       </c>
       <c r="B85" t="str">
-        <v>Mefenoxam</v>
+        <v>Flusilazole</v>
       </c>
       <c r="C85" t="str">
         <v/>
@@ -2109,10 +2109,10 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>metalaxyl</v>
+        <v>flutriafol</v>
       </c>
       <c r="B86" t="str">
-        <v>Metalaxyl</v>
+        <v>Flutriafol</v>
       </c>
       <c r="C86" t="str">
         <v/>
@@ -2129,10 +2129,10 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>methacrifos</v>
+        <v>heptachlor</v>
       </c>
       <c r="B87" t="str">
-        <v>Methacrifos</v>
+        <v>Heptachlor</v>
       </c>
       <c r="C87" t="str">
         <v/>
@@ -2149,10 +2149,10 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>methanol</v>
+        <v>heptachlor_endo_epoxide_isomer_a</v>
       </c>
       <c r="B88" t="str">
-        <v>Methanol</v>
+        <v>Heptachlor endo-epoxide (isomer A)</v>
       </c>
       <c r="C88" t="str">
         <v/>
@@ -2169,10 +2169,10 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>methidathion</v>
+        <v>heptachlor_exo_epoxide_isomer_b</v>
       </c>
       <c r="B89" t="str">
-        <v>Methidathion</v>
+        <v>Heptachlor exo-epoxide (isomer B)</v>
       </c>
       <c r="C89" t="str">
         <v/>
@@ -2189,10 +2189,10 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>methoxychlor_pp_</v>
+        <v>hexachlorobenzene</v>
       </c>
       <c r="B90" t="str">
-        <v>Methoxychlor, p,p'-</v>
+        <v>Hexachlorobenzene</v>
       </c>
       <c r="C90" t="str">
         <v/>
@@ -2209,10 +2209,10 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>mirex</v>
+        <v>hexaconazole</v>
       </c>
       <c r="B91" t="str">
-        <v>Mirex</v>
+        <v>Hexaconazole</v>
       </c>
       <c r="C91" t="str">
         <v/>
@@ -2229,10 +2229,10 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>molinate</v>
+        <v>imazalil</v>
       </c>
       <c r="B92" t="str">
-        <v>Molinate</v>
+        <v>Imazalil</v>
       </c>
       <c r="C92" t="str">
         <v/>
@@ -2249,10 +2249,10 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>monocrotophos</v>
+        <v>iprobenfos</v>
       </c>
       <c r="B93" t="str">
-        <v>Monocrotophos</v>
+        <v>Iprobenfos</v>
       </c>
       <c r="C93" t="str">
         <v/>
@@ -2269,10 +2269,10 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>nitrothal_isopropyl</v>
+        <v>isodrin</v>
       </c>
       <c r="B94" t="str">
-        <v>Nitrothal-Isopropyl</v>
+        <v>Isodrin</v>
       </c>
       <c r="C94" t="str">
         <v/>
@@ -2289,10 +2289,10 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>omega_3</v>
+        <v>isofenfos_methyl</v>
       </c>
       <c r="B95" t="str">
-        <v>Omega 3</v>
+        <v>Isofenphos methyl</v>
       </c>
       <c r="C95" t="str">
         <v/>
@@ -2301,7 +2301,7 @@
         <v/>
       </c>
       <c r="E95" t="str">
-        <v>g/100g</v>
+        <v>ppb</v>
       </c>
       <c r="F95" t="str">
         <v/>
@@ -2309,10 +2309,10 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>omega_6</v>
+        <v>isofenphos_methyl</v>
       </c>
       <c r="B96" t="str">
-        <v>Omega 6</v>
+        <v>Isofenphos methyl</v>
       </c>
       <c r="C96" t="str">
         <v/>
@@ -2321,7 +2321,7 @@
         <v/>
       </c>
       <c r="E96" t="str">
-        <v>g/100g</v>
+        <v>ppb</v>
       </c>
       <c r="F96" t="str">
         <v/>
@@ -2329,10 +2329,10 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>omega_9</v>
+        <v>kresoxim_methyl</v>
       </c>
       <c r="B97" t="str">
-        <v>Omega 9</v>
+        <v>Kresoxim methyl</v>
       </c>
       <c r="C97" t="str">
         <v/>
@@ -2341,7 +2341,7 @@
         <v/>
       </c>
       <c r="E97" t="str">
-        <v>g/100g</v>
+        <v>ppb</v>
       </c>
       <c r="F97" t="str">
         <v/>
@@ -2349,10 +2349,10 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>omethoate</v>
+        <v>lamda_cyhalothrin</v>
       </c>
       <c r="B98" t="str">
-        <v>Omethoate</v>
+        <v>lamda-Cyhalothrin</v>
       </c>
       <c r="C98" t="str">
         <v/>
@@ -2369,10 +2369,10 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>paclobutrazol</v>
+        <v>lambda_cyhalothrin</v>
       </c>
       <c r="B99" t="str">
-        <v>Paclobutrazol</v>
+        <v>lamda-Cyhalothrin</v>
       </c>
       <c r="C99" t="str">
         <v/>
@@ -2389,10 +2389,10 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>parathion</v>
+        <v>malathion</v>
       </c>
       <c r="B100" t="str">
-        <v>Parathion</v>
+        <v>Malathion</v>
       </c>
       <c r="C100" t="str">
         <v/>
@@ -2409,10 +2409,10 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>parathion_methyl</v>
+        <v>mecarbam</v>
       </c>
       <c r="B101" t="str">
-        <v>Parathion-methyl</v>
+        <v>Mecarbam</v>
       </c>
       <c r="C101" t="str">
         <v/>
@@ -2429,10 +2429,10 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>pendimethalin</v>
+        <v>mefenacet</v>
       </c>
       <c r="B102" t="str">
-        <v>Pendimethalin</v>
+        <v>Mefenacet</v>
       </c>
       <c r="C102" t="str">
         <v/>
@@ -2449,10 +2449,10 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>permethrin_cis</v>
+        <v>mefenoxam</v>
       </c>
       <c r="B103" t="str">
-        <v>Permethrin cis</v>
+        <v>Mefenoxam</v>
       </c>
       <c r="C103" t="str">
         <v/>
@@ -2469,10 +2469,10 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>permethrin_trans</v>
+        <v>metalaxyl</v>
       </c>
       <c r="B104" t="str">
-        <v>Permethrin trans</v>
+        <v>Metalaxyl</v>
       </c>
       <c r="C104" t="str">
         <v/>
@@ -2489,10 +2489,10 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>phenthoate</v>
+        <v>methacrifos</v>
       </c>
       <c r="B105" t="str">
-        <v>Phenthoate</v>
+        <v>Methacrifos</v>
       </c>
       <c r="C105" t="str">
         <v/>
@@ -2509,10 +2509,10 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>phorate</v>
+        <v>methanol</v>
       </c>
       <c r="B106" t="str">
-        <v>Phorate</v>
+        <v>Methanol</v>
       </c>
       <c r="C106" t="str">
         <v/>
@@ -2529,10 +2529,10 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>phosmet</v>
+        <v>methidathion</v>
       </c>
       <c r="B107" t="str">
-        <v>Phosmet</v>
+        <v>Methidathion</v>
       </c>
       <c r="C107" t="str">
         <v/>
@@ -2549,10 +2549,10 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>phosphamidon</v>
+        <v>methoxychlor_p_p</v>
       </c>
       <c r="B108" t="str">
-        <v>Phosphamidon</v>
+        <v>Methoxychlor, p,p'-</v>
       </c>
       <c r="C108" t="str">
         <v/>
@@ -2569,10 +2569,10 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>piperonyl_butoxide</v>
+        <v>methoxychlor_pp_</v>
       </c>
       <c r="B109" t="str">
-        <v>Piperonyl butoxide</v>
+        <v>Methoxychlor, p,p'-</v>
       </c>
       <c r="C109" t="str">
         <v/>
@@ -2589,10 +2589,10 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>pirimiphos_methyl</v>
+        <v>metolachlor</v>
       </c>
       <c r="B110" t="str">
-        <v>Pirimiphos methyl</v>
+        <v>Metolachlor</v>
       </c>
       <c r="C110" t="str">
         <v/>
@@ -2604,15 +2604,15 @@
         <v>ppb</v>
       </c>
       <c r="F110" t="str">
-        <v/>
+        <v>SOP 9.14 USDA</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>profenofos</v>
+        <v>mgk_264</v>
       </c>
       <c r="B111" t="str">
-        <v>Profenofos</v>
+        <v>MGK-264</v>
       </c>
       <c r="C111" t="str">
         <v/>
@@ -2624,15 +2624,15 @@
         <v>ppb</v>
       </c>
       <c r="F111" t="str">
-        <v/>
+        <v>SOP 9.14 USDA</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>propanil</v>
+        <v>mirex</v>
       </c>
       <c r="B112" t="str">
-        <v>Propanil</v>
+        <v>Mirex</v>
       </c>
       <c r="C112" t="str">
         <v/>
@@ -2649,10 +2649,10 @@
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>propiconazole</v>
+        <v>molinate</v>
       </c>
       <c r="B113" t="str">
-        <v>Propiconazole</v>
+        <v>Molinate</v>
       </c>
       <c r="C113" t="str">
         <v/>
@@ -2669,10 +2669,10 @@
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>propoxur</v>
+        <v>monocrotophos</v>
       </c>
       <c r="B114" t="str">
-        <v>Propoxur</v>
+        <v>Monocrotophos</v>
       </c>
       <c r="C114" t="str">
         <v/>
@@ -2689,10 +2689,10 @@
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>quinalphos</v>
+        <v>nitrothal_isopropyl</v>
       </c>
       <c r="B115" t="str">
-        <v>Quinalphos</v>
+        <v>Nitrothal-Isopropyl</v>
       </c>
       <c r="C115" t="str">
         <v/>
@@ -2709,10 +2709,10 @@
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>ronnel_fenchlorphos</v>
+        <v>nonachlor_cis</v>
       </c>
       <c r="B116" t="str">
-        <v>Ronnel (Fenchlorphos)</v>
+        <v>Nonachlor cis</v>
       </c>
       <c r="C116" t="str">
         <v/>
@@ -2724,15 +2724,15 @@
         <v>ppb</v>
       </c>
       <c r="F116" t="str">
-        <v/>
+        <v>SOP 9.14 USDA</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>silafluofen_2</v>
+        <v>nonachlor_trans</v>
       </c>
       <c r="B117" t="str">
-        <v>Silafluofen</v>
+        <v>Nonachlor trans</v>
       </c>
       <c r="C117" t="str">
         <v/>
@@ -2744,15 +2744,15 @@
         <v>ppb</v>
       </c>
       <c r="F117" t="str">
-        <v/>
+        <v>SOP 9.14 USDA</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>silafluofen</v>
+        <v>omega_3</v>
       </c>
       <c r="B118" t="str">
-        <v>Silafluofen</v>
+        <v>Omega 3</v>
       </c>
       <c r="C118" t="str">
         <v/>
@@ -2761,7 +2761,7 @@
         <v/>
       </c>
       <c r="E118" t="str">
-        <v>ppb</v>
+        <v>g/100g</v>
       </c>
       <c r="F118" t="str">
         <v/>
@@ -2769,10 +2769,10 @@
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>simazine</v>
+        <v>omega_6</v>
       </c>
       <c r="B119" t="str">
-        <v>Simazine</v>
+        <v>Omega 6</v>
       </c>
       <c r="C119" t="str">
         <v/>
@@ -2781,7 +2781,7 @@
         <v/>
       </c>
       <c r="E119" t="str">
-        <v>ppb</v>
+        <v>g/100g</v>
       </c>
       <c r="F119" t="str">
         <v/>
@@ -2789,10 +2789,10 @@
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>tebuconazole</v>
+        <v>omega_9</v>
       </c>
       <c r="B120" t="str">
-        <v>Tebuconazole</v>
+        <v>Omega 9</v>
       </c>
       <c r="C120" t="str">
         <v/>
@@ -2801,7 +2801,7 @@
         <v/>
       </c>
       <c r="E120" t="str">
-        <v>ppb</v>
+        <v>g/100g</v>
       </c>
       <c r="F120" t="str">
         <v/>
@@ -2809,10 +2809,10 @@
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>tebufenpyrad</v>
+        <v>omethoate</v>
       </c>
       <c r="B121" t="str">
-        <v>Tebufenpyrad</v>
+        <v>Omethoate</v>
       </c>
       <c r="C121" t="str">
         <v/>
@@ -2829,10 +2829,10 @@
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>tebuthiuron</v>
+        <v>paclobutrazol</v>
       </c>
       <c r="B122" t="str">
-        <v>Tebuthiuron</v>
+        <v>Paclobutrazol</v>
       </c>
       <c r="C122" t="str">
         <v/>
@@ -2849,10 +2849,10 @@
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>tefluthrin</v>
+        <v>parathion</v>
       </c>
       <c r="B123" t="str">
-        <v>Tefluthrin</v>
+        <v>Parathion</v>
       </c>
       <c r="C123" t="str">
         <v/>
@@ -2869,10 +2869,10 @@
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>tetraconazole</v>
+        <v>parathion_ethyl</v>
       </c>
       <c r="B124" t="str">
-        <v>Tetraconazole</v>
+        <v>Parathion</v>
       </c>
       <c r="C124" t="str">
         <v/>
@@ -2889,10 +2889,10 @@
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>thiabendazole</v>
+        <v>parathion_methyl</v>
       </c>
       <c r="B125" t="str">
-        <v>Thiabendazole</v>
+        <v>Parathion-methyl</v>
       </c>
       <c r="C125" t="str">
         <v/>
@@ -2909,10 +2909,10 @@
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>sfa_total</v>
+        <v>pendimethalin</v>
       </c>
       <c r="B126" t="str">
-        <v>Tổng Béo bão hòa (SFA)</v>
+        <v>Pendimethalin</v>
       </c>
       <c r="C126" t="str">
         <v/>
@@ -2921,7 +2921,7 @@
         <v/>
       </c>
       <c r="E126" t="str">
-        <v>g/100g</v>
+        <v>ppb</v>
       </c>
       <c r="F126" t="str">
         <v/>
@@ -2929,10 +2929,10 @@
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>ufa_total</v>
+        <v>pentachloroaniline_pca</v>
       </c>
       <c r="B127" t="str">
-        <v>Tổng Béo không bão hòa (UFA)</v>
+        <v>Pentachloroaniline (PCA)</v>
       </c>
       <c r="C127" t="str">
         <v/>
@@ -2941,18 +2941,18 @@
         <v/>
       </c>
       <c r="E127" t="str">
-        <v>g/100g</v>
+        <v>ppb</v>
       </c>
       <c r="F127" t="str">
-        <v/>
+        <v>SOP 9.14 USDA</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>tralomethrin</v>
+        <v>pentachlorobenzene_pcb</v>
       </c>
       <c r="B128" t="str">
-        <v>Tralomethrin</v>
+        <v>Pentachlorobenzene (PCB)</v>
       </c>
       <c r="C128" t="str">
         <v/>
@@ -2964,15 +2964,15 @@
         <v>ppb</v>
       </c>
       <c r="F128" t="str">
-        <v/>
+        <v>SOP 9.14 USDA</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>triadimenol</v>
+        <v>permethrin_cis</v>
       </c>
       <c r="B129" t="str">
-        <v>Triadimenol</v>
+        <v>Permethrin cis</v>
       </c>
       <c r="C129" t="str">
         <v/>
@@ -2989,10 +2989,10 @@
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>triazophos</v>
+        <v>permethrin_trans</v>
       </c>
       <c r="B130" t="str">
-        <v>Triazophos</v>
+        <v>Permethrin trans</v>
       </c>
       <c r="C130" t="str">
         <v/>
@@ -3009,10 +3009,10 @@
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>trichlorfondipterexdichlorvos</v>
+        <v>phenthoate</v>
       </c>
       <c r="B131" t="str">
-        <v>Trichlorfon(Dipterex)/Dichlorvos</v>
+        <v>Phenthoate</v>
       </c>
       <c r="C131" t="str">
         <v/>
@@ -3029,10 +3029,10 @@
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>tricyclazole</v>
+        <v>phorate</v>
       </c>
       <c r="B132" t="str">
-        <v>Tricyclazole</v>
+        <v>Phorate</v>
       </c>
       <c r="C132" t="str">
         <v/>
@@ -3049,10 +3049,10 @@
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>trifluralin</v>
+        <v>phosmet</v>
       </c>
       <c r="B133" t="str">
-        <v>Trifluralin</v>
+        <v>Phosmet</v>
       </c>
       <c r="C133" t="str">
         <v/>
@@ -3069,10 +3069,10 @@
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>uniconazole</v>
+        <v>phosphamidon</v>
       </c>
       <c r="B134" t="str">
-        <v>Uniconazole</v>
+        <v>Phosphamidon</v>
       </c>
       <c r="C134" t="str">
         <v/>
@@ -3089,10 +3089,10 @@
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>vamidothion</v>
+        <v>piperonyl_butoxide</v>
       </c>
       <c r="B135" t="str">
-        <v>Vamidothion</v>
+        <v>Piperonyl butoxide</v>
       </c>
       <c r="C135" t="str">
         <v/>
@@ -3109,27 +3109,627 @@
     </row>
     <row r="136">
       <c r="A136" t="str">
+        <v>pirimiphos_methyl</v>
+      </c>
+      <c r="B136" t="str">
+        <v>Pirimiphos methyl</v>
+      </c>
+      <c r="C136" t="str">
+        <v/>
+      </c>
+      <c r="D136" t="str">
+        <v/>
+      </c>
+      <c r="E136" t="str">
+        <v>ppb</v>
+      </c>
+      <c r="F136" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="str">
+        <v>pirimifos_methyl</v>
+      </c>
+      <c r="B137" t="str">
+        <v>Pirimiphos methyl</v>
+      </c>
+      <c r="C137" t="str">
+        <v/>
+      </c>
+      <c r="D137" t="str">
+        <v/>
+      </c>
+      <c r="E137" t="str">
+        <v>ppb</v>
+      </c>
+      <c r="F137" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="str">
+        <v>profenofos</v>
+      </c>
+      <c r="B138" t="str">
+        <v>Profenofos</v>
+      </c>
+      <c r="C138" t="str">
+        <v/>
+      </c>
+      <c r="D138" t="str">
+        <v/>
+      </c>
+      <c r="E138" t="str">
+        <v>ppb</v>
+      </c>
+      <c r="F138" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="str">
+        <v>pronamide</v>
+      </c>
+      <c r="B139" t="str">
+        <v>Pronamide</v>
+      </c>
+      <c r="C139" t="str">
+        <v/>
+      </c>
+      <c r="D139" t="str">
+        <v/>
+      </c>
+      <c r="E139" t="str">
+        <v>ppb</v>
+      </c>
+      <c r="F139" t="str">
+        <v>SOP 9.14 USDA</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="str">
+        <v>propanil</v>
+      </c>
+      <c r="B140" t="str">
+        <v>Propanil</v>
+      </c>
+      <c r="C140" t="str">
+        <v/>
+      </c>
+      <c r="D140" t="str">
+        <v/>
+      </c>
+      <c r="E140" t="str">
+        <v>ppb</v>
+      </c>
+      <c r="F140" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="str">
+        <v>propiconazole</v>
+      </c>
+      <c r="B141" t="str">
+        <v>Propiconazole</v>
+      </c>
+      <c r="C141" t="str">
+        <v/>
+      </c>
+      <c r="D141" t="str">
+        <v/>
+      </c>
+      <c r="E141" t="str">
+        <v>ppb</v>
+      </c>
+      <c r="F141" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="str">
+        <v>propoxur</v>
+      </c>
+      <c r="B142" t="str">
+        <v>Propoxur</v>
+      </c>
+      <c r="C142" t="str">
+        <v/>
+      </c>
+      <c r="D142" t="str">
+        <v/>
+      </c>
+      <c r="E142" t="str">
+        <v>ppb</v>
+      </c>
+      <c r="F142" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="str">
+        <v>quinalphos</v>
+      </c>
+      <c r="B143" t="str">
+        <v>Quinalphos</v>
+      </c>
+      <c r="C143" t="str">
+        <v/>
+      </c>
+      <c r="D143" t="str">
+        <v/>
+      </c>
+      <c r="E143" t="str">
+        <v>ppb</v>
+      </c>
+      <c r="F143" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="str">
+        <v>ronnel_fenchlorphos</v>
+      </c>
+      <c r="B144" t="str">
+        <v>Ronnel (Fenchlorphos)</v>
+      </c>
+      <c r="C144" t="str">
+        <v/>
+      </c>
+      <c r="D144" t="str">
+        <v/>
+      </c>
+      <c r="E144" t="str">
+        <v>ppb</v>
+      </c>
+      <c r="F144" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="str">
+        <v>silafluofen_2</v>
+      </c>
+      <c r="B145" t="str">
+        <v>Silafluofen</v>
+      </c>
+      <c r="C145" t="str">
+        <v/>
+      </c>
+      <c r="D145" t="str">
+        <v/>
+      </c>
+      <c r="E145" t="str">
+        <v>ppb</v>
+      </c>
+      <c r="F145" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="str">
+        <v>silafluofen</v>
+      </c>
+      <c r="B146" t="str">
+        <v>Silafluofen</v>
+      </c>
+      <c r="C146" t="str">
+        <v/>
+      </c>
+      <c r="D146" t="str">
+        <v/>
+      </c>
+      <c r="E146" t="str">
+        <v>ppb</v>
+      </c>
+      <c r="F146" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="str">
+        <v>simazine</v>
+      </c>
+      <c r="B147" t="str">
+        <v>Simazine</v>
+      </c>
+      <c r="C147" t="str">
+        <v/>
+      </c>
+      <c r="D147" t="str">
+        <v/>
+      </c>
+      <c r="E147" t="str">
+        <v>ppb</v>
+      </c>
+      <c r="F147" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="str">
+        <v>tebuconazole</v>
+      </c>
+      <c r="B148" t="str">
+        <v>Tebuconazole</v>
+      </c>
+      <c r="C148" t="str">
+        <v/>
+      </c>
+      <c r="D148" t="str">
+        <v/>
+      </c>
+      <c r="E148" t="str">
+        <v>ppb</v>
+      </c>
+      <c r="F148" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="str">
+        <v>tebufenpyrad</v>
+      </c>
+      <c r="B149" t="str">
+        <v>Tebufenpyrad</v>
+      </c>
+      <c r="C149" t="str">
+        <v/>
+      </c>
+      <c r="D149" t="str">
+        <v/>
+      </c>
+      <c r="E149" t="str">
+        <v>ppb</v>
+      </c>
+      <c r="F149" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="str">
+        <v>tebuthiuron</v>
+      </c>
+      <c r="B150" t="str">
+        <v>Tebuthiuron</v>
+      </c>
+      <c r="C150" t="str">
+        <v/>
+      </c>
+      <c r="D150" t="str">
+        <v/>
+      </c>
+      <c r="E150" t="str">
+        <v>ppb</v>
+      </c>
+      <c r="F150" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="str">
+        <v>tefluthrin</v>
+      </c>
+      <c r="B151" t="str">
+        <v>Tefluthrin</v>
+      </c>
+      <c r="C151" t="str">
+        <v/>
+      </c>
+      <c r="D151" t="str">
+        <v/>
+      </c>
+      <c r="E151" t="str">
+        <v>ppb</v>
+      </c>
+      <c r="F151" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="str">
+        <v>tetraconazole</v>
+      </c>
+      <c r="B152" t="str">
+        <v>Tetraconazole</v>
+      </c>
+      <c r="C152" t="str">
+        <v/>
+      </c>
+      <c r="D152" t="str">
+        <v/>
+      </c>
+      <c r="E152" t="str">
+        <v>ppb</v>
+      </c>
+      <c r="F152" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="str">
+        <v>thiabendazole</v>
+      </c>
+      <c r="B153" t="str">
+        <v>Thiabendazole</v>
+      </c>
+      <c r="C153" t="str">
+        <v/>
+      </c>
+      <c r="D153" t="str">
+        <v/>
+      </c>
+      <c r="E153" t="str">
+        <v>ppb</v>
+      </c>
+      <c r="F153" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="str">
+        <v>tổng_béo_bão_hòa_(sfa)</v>
+      </c>
+      <c r="B154" t="str">
+        <v>Tổng Béo bão hòa (SFA)</v>
+      </c>
+      <c r="C154" t="str">
+        <v/>
+      </c>
+      <c r="D154" t="str">
+        <v/>
+      </c>
+      <c r="E154" t="str">
+        <v>g/100g</v>
+      </c>
+      <c r="F154" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="str">
+        <v>sfa_total</v>
+      </c>
+      <c r="B155" t="str">
+        <v>Tổng Béo bão hòa (SFA)</v>
+      </c>
+      <c r="C155" t="str">
+        <v/>
+      </c>
+      <c r="D155" t="str">
+        <v/>
+      </c>
+      <c r="E155" t="str">
+        <v>g/100g</v>
+      </c>
+      <c r="F155" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="str">
+        <v>tổng_béo_không_bão_hòa_(ufa)</v>
+      </c>
+      <c r="B156" t="str">
+        <v>Tổng Béo không bão hòa (UFA)</v>
+      </c>
+      <c r="C156" t="str">
+        <v/>
+      </c>
+      <c r="D156" t="str">
+        <v/>
+      </c>
+      <c r="E156" t="str">
+        <v>g/100g</v>
+      </c>
+      <c r="F156" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="str">
+        <v>ufa_total</v>
+      </c>
+      <c r="B157" t="str">
+        <v>Tổng Béo không bão hòa (UFA)</v>
+      </c>
+      <c r="C157" t="str">
+        <v/>
+      </c>
+      <c r="D157" t="str">
+        <v/>
+      </c>
+      <c r="E157" t="str">
+        <v>g/100g</v>
+      </c>
+      <c r="F157" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="str">
+        <v>tralomethrin</v>
+      </c>
+      <c r="B158" t="str">
+        <v>Tralomethrin</v>
+      </c>
+      <c r="C158" t="str">
+        <v/>
+      </c>
+      <c r="D158" t="str">
+        <v/>
+      </c>
+      <c r="E158" t="str">
+        <v>ppb</v>
+      </c>
+      <c r="F158" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="str">
+        <v>triadimenol</v>
+      </c>
+      <c r="B159" t="str">
+        <v>Triadimenol</v>
+      </c>
+      <c r="C159" t="str">
+        <v/>
+      </c>
+      <c r="D159" t="str">
+        <v/>
+      </c>
+      <c r="E159" t="str">
+        <v>ppb</v>
+      </c>
+      <c r="F159" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="str">
+        <v>triazophos</v>
+      </c>
+      <c r="B160" t="str">
+        <v>Triazophos</v>
+      </c>
+      <c r="C160" t="str">
+        <v/>
+      </c>
+      <c r="D160" t="str">
+        <v/>
+      </c>
+      <c r="E160" t="str">
+        <v>ppb</v>
+      </c>
+      <c r="F160" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="str">
+        <v>trichlorfondipterexdichlorvos</v>
+      </c>
+      <c r="B161" t="str">
+        <v>Trichlorfon(Dipterex)/Dichlorvos</v>
+      </c>
+      <c r="C161" t="str">
+        <v/>
+      </c>
+      <c r="D161" t="str">
+        <v/>
+      </c>
+      <c r="E161" t="str">
+        <v>ppb</v>
+      </c>
+      <c r="F161" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="str">
+        <v>tricyclazole</v>
+      </c>
+      <c r="B162" t="str">
+        <v>Tricyclazole</v>
+      </c>
+      <c r="C162" t="str">
+        <v/>
+      </c>
+      <c r="D162" t="str">
+        <v/>
+      </c>
+      <c r="E162" t="str">
+        <v>ppb</v>
+      </c>
+      <c r="F162" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="str">
+        <v>trifluralin</v>
+      </c>
+      <c r="B163" t="str">
+        <v>Trifluralin</v>
+      </c>
+      <c r="C163" t="str">
+        <v/>
+      </c>
+      <c r="D163" t="str">
+        <v/>
+      </c>
+      <c r="E163" t="str">
+        <v>ppb</v>
+      </c>
+      <c r="F163" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="str">
+        <v>uniconazole</v>
+      </c>
+      <c r="B164" t="str">
+        <v>Uniconazole</v>
+      </c>
+      <c r="C164" t="str">
+        <v/>
+      </c>
+      <c r="D164" t="str">
+        <v/>
+      </c>
+      <c r="E164" t="str">
+        <v>ppb</v>
+      </c>
+      <c r="F164" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="str">
+        <v>vamidothion</v>
+      </c>
+      <c r="B165" t="str">
+        <v>Vamidothion</v>
+      </c>
+      <c r="C165" t="str">
+        <v/>
+      </c>
+      <c r="D165" t="str">
+        <v/>
+      </c>
+      <c r="E165" t="str">
+        <v>ppb</v>
+      </c>
+      <c r="F165" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="str">
         <v>vinclozolin</v>
       </c>
-      <c r="B136" t="str">
+      <c r="B166" t="str">
         <v>Vinclozolin</v>
       </c>
-      <c r="C136" t="str">
-        <v/>
-      </c>
-      <c r="D136" t="str">
-        <v/>
-      </c>
-      <c r="E136" t="str">
-        <v>ppb</v>
-      </c>
-      <c r="F136" t="str">
+      <c r="C166" t="str">
+        <v/>
+      </c>
+      <c r="D166" t="str">
+        <v/>
+      </c>
+      <c r="E166" t="str">
+        <v>ppb</v>
+      </c>
+      <c r="F166" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F136"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F166"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: implement standards request management system with kanban and table views
</commit_message>
<xml_diff>
--- a/LIMS_Master_Analytes.xlsx
+++ b/LIMS_Master_Analytes.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F166"/>
+  <dimension ref="A1:F167"/>
   <cols>
     <col min="1" max="1" width="39.83203125" customWidth="1"/>
     <col min="2" max="2" width="39.83203125" customWidth="1"/>
@@ -3009,10 +3009,10 @@
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>phenthoate</v>
+        <v>permethrins</v>
       </c>
       <c r="B131" t="str">
-        <v>Phenthoate</v>
+        <v>Permethrins</v>
       </c>
       <c r="C131" t="str">
         <v/>
@@ -3029,10 +3029,10 @@
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>phorate</v>
+        <v>phenthoate</v>
       </c>
       <c r="B132" t="str">
-        <v>Phorate</v>
+        <v>Phenthoate</v>
       </c>
       <c r="C132" t="str">
         <v/>
@@ -3049,10 +3049,10 @@
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>phosmet</v>
+        <v>phorate</v>
       </c>
       <c r="B133" t="str">
-        <v>Phosmet</v>
+        <v>Phorate</v>
       </c>
       <c r="C133" t="str">
         <v/>
@@ -3069,10 +3069,10 @@
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>phosphamidon</v>
+        <v>phosmet</v>
       </c>
       <c r="B134" t="str">
-        <v>Phosphamidon</v>
+        <v>Phosmet</v>
       </c>
       <c r="C134" t="str">
         <v/>
@@ -3089,10 +3089,10 @@
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>piperonyl_butoxide</v>
+        <v>phosphamidon</v>
       </c>
       <c r="B135" t="str">
-        <v>Piperonyl butoxide</v>
+        <v>Phosphamidon</v>
       </c>
       <c r="C135" t="str">
         <v/>
@@ -3109,10 +3109,10 @@
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>pirimiphos_methyl</v>
+        <v>piperonyl_butoxide</v>
       </c>
       <c r="B136" t="str">
-        <v>Pirimiphos methyl</v>
+        <v>Piperonyl butoxide</v>
       </c>
       <c r="C136" t="str">
         <v/>
@@ -3129,7 +3129,7 @@
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>pirimifos_methyl</v>
+        <v>pirimiphos_methyl</v>
       </c>
       <c r="B137" t="str">
         <v>Pirimiphos methyl</v>
@@ -3149,10 +3149,10 @@
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>profenofos</v>
+        <v>pirimifos_methyl</v>
       </c>
       <c r="B138" t="str">
-        <v>Profenofos</v>
+        <v>Pirimiphos methyl</v>
       </c>
       <c r="C138" t="str">
         <v/>
@@ -3169,10 +3169,10 @@
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>pronamide</v>
+        <v>profenofos</v>
       </c>
       <c r="B139" t="str">
-        <v>Pronamide</v>
+        <v>Profenofos</v>
       </c>
       <c r="C139" t="str">
         <v/>
@@ -3184,15 +3184,15 @@
         <v>ppb</v>
       </c>
       <c r="F139" t="str">
-        <v>SOP 9.14 USDA</v>
+        <v/>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>propanil</v>
+        <v>pronamide</v>
       </c>
       <c r="B140" t="str">
-        <v>Propanil</v>
+        <v>Pronamide</v>
       </c>
       <c r="C140" t="str">
         <v/>
@@ -3204,15 +3204,15 @@
         <v>ppb</v>
       </c>
       <c r="F140" t="str">
-        <v/>
+        <v>SOP 9.14 USDA</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>propiconazole</v>
+        <v>propanil</v>
       </c>
       <c r="B141" t="str">
-        <v>Propiconazole</v>
+        <v>Propanil</v>
       </c>
       <c r="C141" t="str">
         <v/>
@@ -3229,10 +3229,10 @@
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>propoxur</v>
+        <v>propiconazole</v>
       </c>
       <c r="B142" t="str">
-        <v>Propoxur</v>
+        <v>Propiconazole</v>
       </c>
       <c r="C142" t="str">
         <v/>
@@ -3249,10 +3249,10 @@
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>quinalphos</v>
+        <v>propoxur</v>
       </c>
       <c r="B143" t="str">
-        <v>Quinalphos</v>
+        <v>Propoxur</v>
       </c>
       <c r="C143" t="str">
         <v/>
@@ -3269,10 +3269,10 @@
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v>ronnel_fenchlorphos</v>
+        <v>quinalphos</v>
       </c>
       <c r="B144" t="str">
-        <v>Ronnel (Fenchlorphos)</v>
+        <v>Quinalphos</v>
       </c>
       <c r="C144" t="str">
         <v/>
@@ -3289,10 +3289,10 @@
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>silafluofen_2</v>
+        <v>ronnel_fenchlorphos</v>
       </c>
       <c r="B145" t="str">
-        <v>Silafluofen</v>
+        <v>Ronnel (Fenchlorphos)</v>
       </c>
       <c r="C145" t="str">
         <v/>
@@ -3309,7 +3309,7 @@
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v>silafluofen</v>
+        <v>silafluofen_2</v>
       </c>
       <c r="B146" t="str">
         <v>Silafluofen</v>
@@ -3329,10 +3329,10 @@
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>simazine</v>
+        <v>silafluofen</v>
       </c>
       <c r="B147" t="str">
-        <v>Simazine</v>
+        <v>Silafluofen</v>
       </c>
       <c r="C147" t="str">
         <v/>
@@ -3349,10 +3349,10 @@
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>tebuconazole</v>
+        <v>simazine</v>
       </c>
       <c r="B148" t="str">
-        <v>Tebuconazole</v>
+        <v>Simazine</v>
       </c>
       <c r="C148" t="str">
         <v/>
@@ -3369,10 +3369,10 @@
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>tebufenpyrad</v>
+        <v>tebuconazole</v>
       </c>
       <c r="B149" t="str">
-        <v>Tebufenpyrad</v>
+        <v>Tebuconazole</v>
       </c>
       <c r="C149" t="str">
         <v/>
@@ -3389,10 +3389,10 @@
     </row>
     <row r="150">
       <c r="A150" t="str">
-        <v>tebuthiuron</v>
+        <v>tebufenpyrad</v>
       </c>
       <c r="B150" t="str">
-        <v>Tebuthiuron</v>
+        <v>Tebufenpyrad</v>
       </c>
       <c r="C150" t="str">
         <v/>
@@ -3409,10 +3409,10 @@
     </row>
     <row r="151">
       <c r="A151" t="str">
-        <v>tefluthrin</v>
+        <v>tebuthiuron</v>
       </c>
       <c r="B151" t="str">
-        <v>Tefluthrin</v>
+        <v>Tebuthiuron</v>
       </c>
       <c r="C151" t="str">
         <v/>
@@ -3429,10 +3429,10 @@
     </row>
     <row r="152">
       <c r="A152" t="str">
-        <v>tetraconazole</v>
+        <v>tefluthrin</v>
       </c>
       <c r="B152" t="str">
-        <v>Tetraconazole</v>
+        <v>Tefluthrin</v>
       </c>
       <c r="C152" t="str">
         <v/>
@@ -3449,10 +3449,10 @@
     </row>
     <row r="153">
       <c r="A153" t="str">
-        <v>thiabendazole</v>
+        <v>tetraconazole</v>
       </c>
       <c r="B153" t="str">
-        <v>Thiabendazole</v>
+        <v>Tetraconazole</v>
       </c>
       <c r="C153" t="str">
         <v/>
@@ -3469,10 +3469,10 @@
     </row>
     <row r="154">
       <c r="A154" t="str">
-        <v>tổng_béo_bão_hòa_(sfa)</v>
+        <v>thiabendazole</v>
       </c>
       <c r="B154" t="str">
-        <v>Tổng Béo bão hòa (SFA)</v>
+        <v>Thiabendazole</v>
       </c>
       <c r="C154" t="str">
         <v/>
@@ -3481,7 +3481,7 @@
         <v/>
       </c>
       <c r="E154" t="str">
-        <v>g/100g</v>
+        <v>ppb</v>
       </c>
       <c r="F154" t="str">
         <v/>
@@ -3489,7 +3489,7 @@
     </row>
     <row r="155">
       <c r="A155" t="str">
-        <v>sfa_total</v>
+        <v>tổng_béo_bão_hòa_(sfa)</v>
       </c>
       <c r="B155" t="str">
         <v>Tổng Béo bão hòa (SFA)</v>
@@ -3509,10 +3509,10 @@
     </row>
     <row r="156">
       <c r="A156" t="str">
-        <v>tổng_béo_không_bão_hòa_(ufa)</v>
+        <v>sfa_total</v>
       </c>
       <c r="B156" t="str">
-        <v>Tổng Béo không bão hòa (UFA)</v>
+        <v>Tổng Béo bão hòa (SFA)</v>
       </c>
       <c r="C156" t="str">
         <v/>
@@ -3529,7 +3529,7 @@
     </row>
     <row r="157">
       <c r="A157" t="str">
-        <v>ufa_total</v>
+        <v>tổng_béo_không_bão_hòa_(ufa)</v>
       </c>
       <c r="B157" t="str">
         <v>Tổng Béo không bão hòa (UFA)</v>
@@ -3549,10 +3549,10 @@
     </row>
     <row r="158">
       <c r="A158" t="str">
-        <v>tralomethrin</v>
+        <v>ufa_total</v>
       </c>
       <c r="B158" t="str">
-        <v>Tralomethrin</v>
+        <v>Tổng Béo không bão hòa (UFA)</v>
       </c>
       <c r="C158" t="str">
         <v/>
@@ -3561,7 +3561,7 @@
         <v/>
       </c>
       <c r="E158" t="str">
-        <v>ppb</v>
+        <v>g/100g</v>
       </c>
       <c r="F158" t="str">
         <v/>
@@ -3569,10 +3569,10 @@
     </row>
     <row r="159">
       <c r="A159" t="str">
-        <v>triadimenol</v>
+        <v>tralomethrin</v>
       </c>
       <c r="B159" t="str">
-        <v>Triadimenol</v>
+        <v>Tralomethrin</v>
       </c>
       <c r="C159" t="str">
         <v/>
@@ -3589,10 +3589,10 @@
     </row>
     <row r="160">
       <c r="A160" t="str">
-        <v>triazophos</v>
+        <v>triadimenol</v>
       </c>
       <c r="B160" t="str">
-        <v>Triazophos</v>
+        <v>Triadimenol</v>
       </c>
       <c r="C160" t="str">
         <v/>
@@ -3609,10 +3609,10 @@
     </row>
     <row r="161">
       <c r="A161" t="str">
-        <v>trichlorfondipterexdichlorvos</v>
+        <v>triazophos</v>
       </c>
       <c r="B161" t="str">
-        <v>Trichlorfon(Dipterex)/Dichlorvos</v>
+        <v>Triazophos</v>
       </c>
       <c r="C161" t="str">
         <v/>
@@ -3629,10 +3629,10 @@
     </row>
     <row r="162">
       <c r="A162" t="str">
-        <v>tricyclazole</v>
+        <v>trichlorfondipterexdichlorvos</v>
       </c>
       <c r="B162" t="str">
-        <v>Tricyclazole</v>
+        <v>Trichlorfon(Dipterex)/Dichlorvos</v>
       </c>
       <c r="C162" t="str">
         <v/>
@@ -3649,10 +3649,10 @@
     </row>
     <row r="163">
       <c r="A163" t="str">
-        <v>trifluralin</v>
+        <v>tricyclazole</v>
       </c>
       <c r="B163" t="str">
-        <v>Trifluralin</v>
+        <v>Tricyclazole</v>
       </c>
       <c r="C163" t="str">
         <v/>
@@ -3669,10 +3669,10 @@
     </row>
     <row r="164">
       <c r="A164" t="str">
-        <v>uniconazole</v>
+        <v>trifluralin</v>
       </c>
       <c r="B164" t="str">
-        <v>Uniconazole</v>
+        <v>Trifluralin</v>
       </c>
       <c r="C164" t="str">
         <v/>
@@ -3689,10 +3689,10 @@
     </row>
     <row r="165">
       <c r="A165" t="str">
-        <v>vamidothion</v>
+        <v>uniconazole</v>
       </c>
       <c r="B165" t="str">
-        <v>Vamidothion</v>
+        <v>Uniconazole</v>
       </c>
       <c r="C165" t="str">
         <v/>
@@ -3709,27 +3709,47 @@
     </row>
     <row r="166">
       <c r="A166" t="str">
+        <v>vamidothion</v>
+      </c>
+      <c r="B166" t="str">
+        <v>Vamidothion</v>
+      </c>
+      <c r="C166" t="str">
+        <v/>
+      </c>
+      <c r="D166" t="str">
+        <v/>
+      </c>
+      <c r="E166" t="str">
+        <v>ppb</v>
+      </c>
+      <c r="F166" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="str">
         <v>vinclozolin</v>
       </c>
-      <c r="B166" t="str">
+      <c r="B167" t="str">
         <v>Vinclozolin</v>
       </c>
-      <c r="C166" t="str">
-        <v/>
-      </c>
-      <c r="D166" t="str">
-        <v/>
-      </c>
-      <c r="E166" t="str">
-        <v>ppb</v>
-      </c>
-      <c r="F166" t="str">
+      <c r="C167" t="str">
+        <v/>
+      </c>
+      <c r="D167" t="str">
+        <v/>
+      </c>
+      <c r="E167" t="str">
+        <v>ppb</v>
+      </c>
+      <c r="F167" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F166"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F167"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>